<commit_message>
1. Unified 4-Column Layout (Matches Super Admin)
2. Coaches Must Self-Register via Partner Link
3. Instant Search Bars
4. Click-to-Sort Columns
</commit_message>
<xml_diff>
--- a/Commission_Apparel_Financial_Test_Sheet.xlsx
+++ b/Commission_Apparel_Financial_Test_Sheet.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Financial Test Sheet" sheetId="1" r:id="rId1"/>
+    <sheet name="Financial Test Matrix" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,24 +397,27 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K14"/>
+  <dimension ref="A1:N22"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="16.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="20.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="38.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="11.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
+    <col min="9" max="9" width="15.83203125" customWidth="1"/>
+    <col min="10" max="10" width="11.83203125" customWidth="1"/>
+    <col min="11" max="11" width="19.83203125" customWidth="1"/>
+    <col min="12" max="12" width="17.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Commission Apparel - Financial &amp; Mathematical Test Matrix</v>
+        <v>Commission Apparel - Financial &amp; Mathematical Test Matrix (Aligned with Staging Seeder)</v>
       </c>
       <c r="B1" t="str">
         <v/>
@@ -444,12 +447,15 @@
         <v/>
       </c>
       <c r="K1" t="str">
+        <v/>
+      </c>
+      <c r="L1" t="str">
         <v/>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Formulas used: Net Margin = MAX(0, Gross - (Mfg + Tariff + Fees)), Rep Earned = Margin * Rate, Company Net = Margin - Rep Earned</v>
+        <v>Seeder File: database/seeders/FinancialTestScenarioSeeder.php</v>
       </c>
       <c r="B2" t="str">
         <v/>
@@ -479,12 +485,15 @@
         <v/>
       </c>
       <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
         <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>⚡ NOTE: Staging Stripe is in Sandbox Mode. Use Test Card: 4242 4242 4242 4242 | Exp: Any future (e.g. 12/28) | CVC: 123 | Zip: 90210</v>
+        <v>Formula Engine: Net Margin = MAX(0, Gross - (Mfg + Tariff + Deductions)) | Rep Earned = Margin * Rate | Company Net = Margin - Rep Earned</v>
       </c>
       <c r="B3" t="str">
         <v/>
@@ -516,325 +525,675 @@
       <c r="K3" t="str">
         <v/>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Case ID</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Scenario Description</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Retail Gross ($)</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Mfg Cost ($)</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Tariff ($)</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Fees / Fundraising ($)</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Net Margin ($)</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Rep Rate</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Rep Commission ($)</v>
-      </c>
-      <c r="J5" t="str">
-        <v>Company Net ($)</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Payout Status</v>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>⚡ Staging Stripe Sandbox Card: 4242 4242 4242 4242 | Exp: Any future date (12/28) | CVC: 123 | Zip: 90210</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v/>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>TC-01</v>
+        <v>Case ID</v>
       </c>
       <c r="B6" t="str">
-        <v>Standard Team Store (50/50 split)</v>
-      </c>
-      <c r="C6">
-        <v>1200</v>
-      </c>
-      <c r="D6">
-        <v>600</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-      <c r="G6">
-        <f>MAX(0, C6-(D6+E6+F6))</f>
-      </c>
-      <c r="H6">
-        <v>0.5</v>
-      </c>
-      <c r="I6">
-        <f>G6*H6</f>
-      </c>
-      <c r="J6">
-        <f>G6-I6</f>
+        <v>Athlete Name</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Order Item Name</v>
+      </c>
+      <c r="D6" t="str">
+        <v>Scenario Description</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Retail Gross ($)</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Mfg Cost ($)</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Tariff ($)</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Fees / Fundraising ($)</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Net Margin ($)</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Rep Rate</v>
       </c>
       <c r="K6" t="str">
-        <v>PENDING</v>
+        <v>Rep Commission ($)</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Company Net ($)</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Payout Status</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Seeder Notes</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>TC-02</v>
+        <v>TC-01</v>
       </c>
       <c r="B7" t="str">
-        <v>Tariff Applied (Import deduction)</v>
-      </c>
-      <c r="C7">
-        <v>2500</v>
-      </c>
-      <c r="D7">
-        <v>1100</v>
+        <v>Marcus Vance</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Custom Sublimated Team Uniform Set</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Standard Team Store (50/50 split)</v>
       </c>
       <c r="E7">
-        <v>150</v>
+        <v>1200</v>
       </c>
       <c r="F7">
+        <v>600</v>
+      </c>
+      <c r="G7">
         <v>0</v>
       </c>
-      <c r="G7">
-        <f>MAX(0, C7-(D7+E7+F7))</f>
-      </c>
       <c r="H7">
+        <v>0</v>
+      </c>
+      <c r="I7">
+        <f>MAX(0, E7-(F7+G7+H7))</f>
+      </c>
+      <c r="J7">
         <v>0.5</v>
       </c>
-      <c r="I7">
-        <f>G7*H7</f>
-      </c>
-      <c r="J7">
-        <f>G7-I7</f>
-      </c>
-      <c r="K7" t="str">
+      <c r="K7">
+        <f>I7*J7</f>
+      </c>
+      <c r="L7">
+        <f>I7-K7</f>
+      </c>
+      <c r="M7" t="str">
         <v>PENDING</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Clean 50/50 split on standard team store order.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>TC-03</v>
+        <v>TC-02</v>
       </c>
       <c r="B8" t="str">
-        <v>School Kickback ($5/item fundraising)</v>
-      </c>
-      <c r="C8">
-        <v>3000</v>
-      </c>
-      <c r="D8">
-        <v>1400</v>
+        <v>Jordan Hayes</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Overseas Custom Sublimation Package</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Tariff Applied (Import deduction)</v>
       </c>
       <c r="E8">
+        <v>2500</v>
+      </c>
+      <c r="F8">
+        <v>1100</v>
+      </c>
+      <c r="G8">
+        <v>150</v>
+      </c>
+      <c r="H8">
         <v>0</v>
       </c>
-      <c r="F8">
-        <v>300</v>
-      </c>
-      <c r="G8">
-        <f>MAX(0, C8-(D8+E8+F8))</f>
-      </c>
-      <c r="H8">
+      <c r="I8">
+        <f>MAX(0, E8-(F8+G8+H8))</f>
+      </c>
+      <c r="J8">
         <v>0.5</v>
       </c>
-      <c r="I8">
-        <f>G8*H8</f>
-      </c>
-      <c r="J8">
-        <f>G8-I8</f>
-      </c>
-      <c r="K8" t="str">
-        <v>CLEARED</v>
+      <c r="K8">
+        <f>I8*J8</f>
+      </c>
+      <c r="L8">
+        <f>I8-K8</f>
+      </c>
+      <c r="M8" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Custom overseas sublimation with $150 tariff deduction.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>TC-04</v>
+        <v>TC-03</v>
       </c>
       <c r="B9" t="str">
-        <v>Senior Rep Tier (60% custom rate)</v>
-      </c>
-      <c r="C9">
-        <v>4800</v>
-      </c>
-      <c r="D9">
-        <v>2200</v>
+        <v>Lucas Reyes</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Varsity Fan Wear &amp; Uniform Combo</v>
+      </c>
+      <c r="D9" t="str">
+        <v>School Kickback ($5/item fundraising)</v>
       </c>
       <c r="E9">
-        <v>100</v>
+        <v>3000</v>
       </c>
       <c r="F9">
-        <v>100</v>
+        <v>1400</v>
       </c>
       <c r="G9">
-        <f>MAX(0, C9-(D9+E9+F9))</f>
+        <v>0</v>
       </c>
       <c r="H9">
-        <v>0.6</v>
+        <v>300</v>
       </c>
       <c r="I9">
-        <f>G9*H9</f>
+        <f>MAX(0, E9-(F9+G9+H9))</f>
       </c>
       <c r="J9">
-        <f>G9-I9</f>
-      </c>
-      <c r="K9" t="str">
+        <v>0.5</v>
+      </c>
+      <c r="K9">
+        <f>I9*J9</f>
+      </c>
+      <c r="L9">
+        <f>I9-K9</f>
+      </c>
+      <c r="M9" t="str">
         <v>CLEARED</v>
+      </c>
+      <c r="N9" t="str">
+        <v>School booster club fundraising kickback of $300 deducted.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>TC-05</v>
+        <v>TC-04</v>
       </c>
       <c r="B10" t="str">
-        <v>Junior Rep Tier (40% custom rate)</v>
-      </c>
-      <c r="C10">
-        <v>1500</v>
-      </c>
-      <c r="D10">
-        <v>750</v>
+        <v>Devon Miller</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Championship Club Pack (Senior Tier)</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Senior Rep Tier (60% custom rate)</v>
       </c>
       <c r="E10">
-        <v>0</v>
+        <v>4800</v>
       </c>
       <c r="F10">
-        <v>50</v>
+        <v>2200</v>
       </c>
       <c r="G10">
-        <f>MAX(0, C10-(D10+E10+F10))</f>
+        <v>100</v>
       </c>
       <c r="H10">
-        <v>0.4</v>
+        <v>100</v>
       </c>
       <c r="I10">
-        <f>G10*H10</f>
+        <f>MAX(0, E10-(F10+G10+H10))</f>
       </c>
       <c r="J10">
-        <f>G10-I10</f>
-      </c>
-      <c r="K10" t="str">
-        <v>PAID</v>
+        <v>0.6</v>
+      </c>
+      <c r="K10">
+        <f>I10*J10</f>
+      </c>
+      <c r="L10">
+        <f>I10-K10</f>
+      </c>
+      <c r="M10" t="str">
+        <v>CLEARED</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Senior partner commission tier override at 60.0%.</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>TC-06</v>
+        <v>TC-05</v>
       </c>
       <c r="B11" t="str">
-        <v>Zero-Margin Guard (Costs &gt;= Gross)</v>
-      </c>
-      <c r="C11">
-        <v>500</v>
-      </c>
-      <c r="D11">
-        <v>480</v>
+        <v>Ethan Cruz</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Youth League Practice Pack (Junior Tier)</v>
+      </c>
+      <c r="D11" t="str">
+        <v>Junior Rep Tier (40% custom rate)</v>
       </c>
       <c r="E11">
-        <v>20</v>
+        <v>1500</v>
       </c>
       <c r="F11">
+        <v>750</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
         <v>50</v>
       </c>
-      <c r="G11">
-        <f>MAX(0, C11-(D11+E11+F11))</f>
-      </c>
-      <c r="H11">
-        <v>0.5</v>
-      </c>
       <c r="I11">
-        <f>G11*H11</f>
+        <f>MAX(0, E11-(F11+G11+H11))</f>
       </c>
       <c r="J11">
-        <f>G11-I11</f>
-      </c>
-      <c r="K11" t="str">
-        <v>PENDING</v>
+        <v>0.4</v>
+      </c>
+      <c r="K11">
+        <f>I11*J11</f>
+      </c>
+      <c r="L11">
+        <f>I11-K11</f>
+      </c>
+      <c r="M11" t="str">
+        <v>PAID</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Junior partner referral tier at 40.0%, fully disbursed.</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
+        <v>TC-06</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Liam Walker</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Rushed Prototype Sample Kit</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Zero-Margin Guard (Costs &gt;= Gross)</v>
+      </c>
+      <c r="E12">
+        <v>500</v>
+      </c>
+      <c r="F12">
+        <v>480</v>
+      </c>
+      <c r="G12">
+        <v>20</v>
+      </c>
+      <c r="H12">
+        <v>50</v>
+      </c>
+      <c r="I12">
+        <f>MAX(0, E12-(F12+G12+H12))</f>
+      </c>
+      <c r="J12">
+        <v>0.5</v>
+      </c>
+      <c r="K12">
+        <f>I12*J12</f>
+      </c>
+      <c r="L12">
+        <f>I12-K12</f>
+      </c>
+      <c r="M12" t="str">
+        <v>PENDING</v>
+      </c>
+      <c r="N12" t="str">
+        <v>High sample cost guard test ($550 total costs vs $500 gross). Clamped to $0.00.</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
         <v>TC-07</v>
       </c>
-      <c r="B12" t="str">
+      <c r="B13" t="str">
+        <v>Tyler Brooke</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Regional Travel Program Elite Batch</v>
+      </c>
+      <c r="D13" t="str">
         <v>High-Volume Club Batch (Tariffs &amp; fees)</v>
       </c>
-      <c r="C12">
+      <c r="E13">
         <v>8500</v>
       </c>
-      <c r="D12">
+      <c r="F13">
         <v>3800</v>
       </c>
-      <c r="E12">
+      <c r="G13">
         <v>350</v>
       </c>
-      <c r="F12">
+      <c r="H13">
         <v>250</v>
       </c>
-      <c r="G12">
-        <f>MAX(0, C12-(D12+E12+F12))</f>
-      </c>
-      <c r="H12">
+      <c r="I13">
+        <f>MAX(0, E13-(F13+G13+H13))</f>
+      </c>
+      <c r="J13">
         <v>0.5</v>
       </c>
-      <c r="I12">
-        <f>G12*H12</f>
-      </c>
-      <c r="J12">
-        <f>G12-I12</f>
-      </c>
-      <c r="K12" t="str">
+      <c r="K13">
+        <f>I13*J13</f>
+      </c>
+      <c r="L13">
+        <f>I13-K13</f>
+      </c>
+      <c r="M13" t="str">
         <v>PAID</v>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
+      <c r="N13" t="str">
+        <v>High volume travel club batch, fully cleared and paid out.</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
         <v>TOTALS</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B15" t="str">
+        <v>—</v>
+      </c>
+      <c r="C15" t="str">
+        <v>—</v>
+      </c>
+      <c r="D15" t="str">
         <v>Portfolio Aggregates</v>
       </c>
-      <c r="C14">
-        <f>SUM(C6:C12)</f>
-      </c>
-      <c r="D14">
-        <f>SUM(D6:D12)</f>
-      </c>
-      <c r="E14">
-        <f>SUM(E6:E12)</f>
-      </c>
-      <c r="F14">
-        <f>SUM(F6:F12)</f>
-      </c>
-      <c r="G14">
-        <f>SUM(G6:G12)</f>
-      </c>
-      <c r="H14" t="str">
+      <c r="E15">
+        <f>SUM(E7:E13)</f>
+      </c>
+      <c r="F15">
+        <f>SUM(F7:F13)</f>
+      </c>
+      <c r="G15">
+        <f>SUM(G7:G13)</f>
+      </c>
+      <c r="H15">
+        <f>SUM(H7:H13)</f>
+      </c>
+      <c r="I15">
+        <f>SUM(I7:I13)</f>
+      </c>
+      <c r="J15" t="str">
         <v>—</v>
       </c>
-      <c r="I14">
-        <f>SUM(I6:I12)</f>
-      </c>
-      <c r="J14">
-        <f>SUM(J6:J12)</f>
-      </c>
-      <c r="K14" t="str">
+      <c r="K15">
+        <f>SUM(K7:K13)</f>
+      </c>
+      <c r="L15">
+        <f>SUM(L7:L13)</f>
+      </c>
+      <c r="M15" t="str">
         <v>—</v>
+      </c>
+      <c r="N15" t="str">
+        <v>—</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>STAGING DASHBOARD SUMMARY CARDS CHECKLIST</v>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+      <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
+        <v/>
+      </c>
+      <c r="L17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Metric Card</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Expected Target</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Seeder Test Cases Included</v>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+      <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
+        <v/>
+      </c>
+      <c r="L18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Pending Commission</v>
+      </c>
+      <c r="B19">
+        <v>925</v>
+      </c>
+      <c r="C19" t="str">
+        <v>TC-01 ($300) + TC-02 ($625) + TC-06 ($0)</v>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+      <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
+        <v/>
+      </c>
+      <c r="L19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Cleared Commission</v>
+      </c>
+      <c r="B20">
+        <v>2090</v>
+      </c>
+      <c r="C20" t="str">
+        <v>TC-03 ($650) + TC-04 ($1,440)</v>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+      <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
+        <v/>
+      </c>
+      <c r="L20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Paid Commission</v>
+      </c>
+      <c r="B21">
+        <v>2330</v>
+      </c>
+      <c r="C21" t="str">
+        <v>TC-05 ($280) + TC-07 ($2,050)</v>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+      <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
+        <v/>
+      </c>
+      <c r="L21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Lifetime Commission Earned</v>
+      </c>
+      <c r="B22">
+        <v>5345</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Sum of all 7 test cases</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
+      </c>
+      <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
+        <v/>
+      </c>
+      <c r="L22" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:N22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>